<commit_message>
Added 4 point scan to config
</commit_message>
<xml_diff>
--- a/configs/config_g3p3_b0.xlsx
+++ b/configs/config_g3p3_b0.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nrel-my.sharepoint.com/personal/sletizia_nrel_gov/Documents/Desktop/Main/G3P3/g3p3_lidar_processing/configs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aabraha2\Documents\G3P3\Codes\g3p3_lidar_processing\configs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="13_ncr:1_{04294DC9-DB31-448F-BB95-920AF215A499}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5855D667-D7B5-43CC-92CA-32DBFFC6CA7E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DE379BB-F87D-462F-B9CF-93380031467D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1920" yWindow="1920" windowWidth="18552" windowHeight="10488" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="1" r:id="rId1"/>
@@ -179,7 +179,7 @@
     <t>roof.lidar.z01.a0.\d{8}.\d{1}(?:030|110|150|230|310|350|430|510|550|630|710|750|830|910|950|)\d{2}.user5.nc</t>
   </si>
   <si>
-    <t>3.points</t>
+    <t>4.points</t>
   </si>
 </sst>
 </file>
@@ -357,10 +357,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -788,7 +784,7 @@
         <v>20250416</v>
       </c>
       <c r="L3" s="22">
-        <v>20250416</v>
+        <v>20250430</v>
       </c>
       <c r="M3" s="3"/>
       <c r="N3" s="3"/>
@@ -824,13 +820,13 @@
         <v>20250416</v>
       </c>
       <c r="J4" s="22">
-        <v>20250430</v>
+        <v>20250601</v>
       </c>
       <c r="K4" s="22">
-        <v>20250430</v>
+        <v>20250601</v>
       </c>
       <c r="L4" s="22">
-        <v>20250430</v>
+        <v>20250601</v>
       </c>
       <c r="M4" s="3"/>
       <c r="N4" s="3"/>
@@ -956,7 +952,7 @@
         <v>-0.1</v>
       </c>
       <c r="L7" s="7">
-        <v>1.4</v>
+        <v>0.4</v>
       </c>
       <c r="M7" s="7"/>
       <c r="N7" s="7"/>
@@ -1040,7 +1036,7 @@
         <v>-0.1</v>
       </c>
       <c r="L9" s="7">
-        <v>-0.1</v>
+        <v>-1.2</v>
       </c>
       <c r="M9" s="7"/>
       <c r="N9" s="7"/>
@@ -1082,7 +1078,7 @@
         <v>50</v>
       </c>
       <c r="L10" s="7">
-        <v>0.1</v>
+        <v>1.2</v>
       </c>
       <c r="M10" s="7"/>
       <c r="N10" s="7"/>
@@ -1586,7 +1582,7 @@
         <v>0.1</v>
       </c>
       <c r="L22" s="24">
-        <v>0.1</v>
+        <v>1E-4</v>
       </c>
       <c r="M22" s="13"/>
       <c r="N22" s="13"/>

</xml_diff>